<commit_message>
Code für Latex-tabelle zur analyse der daten geschrieben
</commit_message>
<xml_diff>
--- a/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
+++ b/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D1753C6D-6F34-4E7C-B94D-B14167CAA7E7}"/>
+  <xr:revisionPtr revIDLastSave="31" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0EE37BE-6C99-439D-BD6D-6D41DB675F3C}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16305" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
   <si>
     <r>
       <t xml:space="preserve">März 2026: </t>
@@ -82,24 +82,6 @@
     <t>Gesamt</t>
   </si>
   <si>
-    <t>Einführung in die Theorie, welche Normen es für die Glasproduktion usw. gibt</t>
-  </si>
-  <si>
-    <t>Normungsunterlagen durcharbeiten</t>
-  </si>
-  <si>
-    <t>Nummerischer Ansatz anhand theoretischem Muster</t>
-  </si>
-  <si>
-    <t>Vergleichstest</t>
-  </si>
-  <si>
-    <t>Neues Konzept betreffend Auflagepunkte</t>
-  </si>
-  <si>
-    <t>Erneut neues Konzept betreffend Auflagepunkte</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">März 2026: </t>
     </r>
@@ -114,13 +96,40 @@
     </r>
   </si>
   <si>
+    <t>Einführung in die Theorie, welche Normen es für die Glasproduktion usw. gibt</t>
+  </si>
+  <si>
     <t>Kilometer</t>
   </si>
   <si>
+    <t>Normungsunterlagen durcharbeiten</t>
+  </si>
+  <si>
+    <t>Nummerischer Ansatz anhand theoretischem Muster</t>
+  </si>
+  <si>
+    <t>Vergleichstest</t>
+  </si>
+  <si>
     <t>-</t>
   </si>
   <si>
     <t>Home-Office</t>
+  </si>
+  <si>
+    <t>Neues Konzept betreffend Auflagepunkte</t>
+  </si>
+  <si>
+    <t>Zwischenergebnis - MÄRZ</t>
+  </si>
+  <si>
+    <t>Erneut neues Konzept betreffend Auflagepunkte</t>
+  </si>
+  <si>
+    <t>Analyse der Gravitationsauswirkung auf verschiedene Glasplatten</t>
+  </si>
+  <si>
+    <t>Code zur Speicherung der Analyse Daten geschrieben</t>
   </si>
 </sst>
 </file>
@@ -500,7 +509,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -551,14 +560,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="21" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="46" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="21" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -893,29 +913,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="5" max="5" width="66.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" s="34" t="s">
+    <row r="1" spans="1:19">
+      <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
-      <c r="H1" s="35"/>
-      <c r="I1" s="35"/>
+      <c r="B1" s="44"/>
+      <c r="C1" s="44"/>
+      <c r="D1" s="44"/>
+      <c r="E1" s="44"/>
+      <c r="F1" s="44"/>
+      <c r="G1" s="44"/>
+      <c r="H1" s="44"/>
+      <c r="I1" s="44"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:11" ht="15" thickBot="1">
+    <row r="2" spans="1:19" ht="15">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="2"/>
@@ -928,7 +948,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
     </row>
-    <row r="3" spans="1:11" ht="26.25" thickBot="1">
+    <row r="3" spans="1:19" ht="27.75">
       <c r="A3" s="24" t="s">
         <v>1</v>
       </c>
@@ -957,9 +977,19 @@
         <v>9</v>
       </c>
       <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-    </row>
-    <row r="4" spans="1:11">
+      <c r="K3" s="36" t="s">
+        <v>10</v>
+      </c>
+      <c r="L3" s="37"/>
+      <c r="M3" s="37"/>
+      <c r="N3" s="37"/>
+      <c r="O3" s="37"/>
+      <c r="P3" s="37"/>
+      <c r="Q3" s="37"/>
+      <c r="R3" s="37"/>
+      <c r="S3" s="37"/>
+    </row>
+    <row r="4" spans="1:19" ht="15">
       <c r="A4" s="20">
         <v>46086</v>
       </c>
@@ -973,7 +1003,7 @@
         <v>0.3923611111111111</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" s="6">
         <v>0.54861111111111105</v>
@@ -990,9 +1020,14 @@
         <v>0.36805555555555552</v>
       </c>
       <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="K4" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="L4" s="29" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="15">
       <c r="A5" s="16">
         <v>46087</v>
       </c>
@@ -1006,7 +1041,7 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F5" s="3">
         <v>0.54166666666666663</v>
@@ -1023,9 +1058,14 @@
         <v>0.39583333333333326</v>
       </c>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-    </row>
-    <row r="6" spans="1:11">
+      <c r="K5" s="8">
+        <v>46086</v>
+      </c>
+      <c r="L5" s="31">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" ht="15">
       <c r="A6" s="16">
         <v>46093</v>
       </c>
@@ -1039,7 +1079,7 @@
         <v>0.38541666666666669</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F6" s="3">
         <v>0.58333333333333337</v>
@@ -1056,9 +1096,14 @@
         <v>0.36458333333333343</v>
       </c>
       <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-    </row>
-    <row r="7" spans="1:11" ht="15" thickBot="1">
+      <c r="K6" s="16">
+        <v>46087</v>
+      </c>
+      <c r="L6" s="32">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" ht="15">
       <c r="A7" s="18">
         <v>46095</v>
       </c>
@@ -1072,7 +1117,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="E7" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F7" s="5">
         <v>0.54166666666666663</v>
@@ -1089,9 +1134,14 @@
         <v>0.27083333333333326</v>
       </c>
       <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-    </row>
-    <row r="8" spans="1:11">
+      <c r="K7" s="16">
+        <v>46093</v>
+      </c>
+      <c r="L7" s="32">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="15">
       <c r="A8" s="8">
         <v>46100</v>
       </c>
@@ -1105,7 +1155,7 @@
         <v>0.3125</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F8" s="9">
         <v>0.51041666666666663</v>
@@ -1122,9 +1172,14 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="1:11" ht="15" thickBot="1">
+      <c r="K8" s="16">
+        <v>46095</v>
+      </c>
+      <c r="L8" s="32">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="15">
       <c r="A9" s="12">
         <v>46100</v>
       </c>
@@ -1138,7 +1193,7 @@
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F9" s="22">
         <v>0</v>
@@ -1155,9 +1210,14 @@
         <v>4.166666666666663E-2</v>
       </c>
       <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-    </row>
-    <row r="10" spans="1:11" ht="15" thickBot="1">
+      <c r="K9" s="16">
+        <v>46100</v>
+      </c>
+      <c r="L9" s="32">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="15">
       <c r="A10" s="20">
         <v>46101</v>
       </c>
@@ -1171,7 +1231,7 @@
         <v>0.29166666666666669</v>
       </c>
       <c r="E10" s="7" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F10" s="22">
         <v>0</v>
@@ -1188,9 +1248,17 @@
         <v>0.25</v>
       </c>
       <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-    </row>
-    <row r="11" spans="1:11">
+      <c r="K10" s="16">
+        <v>46101</v>
+      </c>
+      <c r="L10" s="32" t="s">
+        <v>16</v>
+      </c>
+      <c r="M10" s="30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="15">
       <c r="A11" s="16">
         <v>46107</v>
       </c>
@@ -1204,7 +1272,7 @@
         <v>0.3923611111111111</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F11" s="3">
         <v>0.54861111111111116</v>
@@ -1221,9 +1289,14 @@
         <v>0.36805555555555564</v>
       </c>
       <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-    </row>
-    <row r="12" spans="1:11" ht="15" thickBot="1">
+      <c r="K11" s="16">
+        <v>46107</v>
+      </c>
+      <c r="L11" s="32">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="15">
       <c r="A12" s="12">
         <v>46108</v>
       </c>
@@ -1237,7 +1310,7 @@
         <v>0.41666666666666669</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="F12" s="13">
         <v>0.51041666666666663</v>
@@ -1254,62 +1327,99 @@
         <v>0.39583333333333326</v>
       </c>
       <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-    </row>
-    <row r="13" spans="1:11" ht="15" thickBot="1">
-      <c r="A13" s="36">
-        <v>46117</v>
-      </c>
-      <c r="B13" s="37">
-        <v>0.38541666666666669</v>
-      </c>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
+      <c r="K12" s="12">
+        <v>46108</v>
+      </c>
+      <c r="L12" s="33" t="s">
+        <v>16</v>
+      </c>
+      <c r="M12" s="30" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="15">
+      <c r="A13" t="s">
+        <v>19</v>
+      </c>
       <c r="I13" s="23">
         <f>SUM(I4:I12)</f>
         <v>2.7465277777777777</v>
       </c>
       <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-    </row>
-    <row r="14" spans="1:11">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
+    </row>
+    <row r="14" spans="1:19" ht="15">
+      <c r="A14" s="34">
+        <v>46117</v>
+      </c>
+      <c r="B14" s="35">
+        <v>0.38541666666666669</v>
+      </c>
+      <c r="C14" s="38">
+        <v>0.71527777777777779</v>
+      </c>
+      <c r="D14" s="38">
+        <v>0.3298611111111111</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="40">
+        <v>0.5625</v>
+      </c>
+      <c r="G14" s="38">
+        <v>0.57986111111111116</v>
+      </c>
+      <c r="H14" s="39">
+        <v>1.7361111111111112E-2</v>
+      </c>
+      <c r="I14" s="38">
+        <v>0.3125</v>
+      </c>
       <c r="J14" s="2"/>
-      <c r="K14" s="2"/>
-    </row>
-    <row r="15" spans="1:11">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
+    </row>
+    <row r="15" spans="1:19" ht="15">
+      <c r="A15" s="34">
+        <v>46117</v>
+      </c>
+      <c r="B15" s="41">
+        <v>0.45833333333333331</v>
+      </c>
+      <c r="C15" s="42">
+        <v>5.5555555555555552E-2</v>
+      </c>
+      <c r="D15" s="38">
+        <v>9.7222222222222224E-2</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F15" s="22">
+        <v>0</v>
+      </c>
+      <c r="G15" s="22">
+        <v>0</v>
+      </c>
+      <c r="H15" s="38">
+        <v>0</v>
+      </c>
+      <c r="I15" s="38">
+        <v>9.7222222222222224E-2</v>
+      </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
-    <row r="16" spans="1:11">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
+    <row r="16" spans="1:19" ht="15">
+      <c r="A16" s="34">
+        <v>46118</v>
+      </c>
+      <c r="B16" s="35">
+        <v>0.41666666666666669</v>
+      </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="E16" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
@@ -1317,101 +1427,22 @@
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="18" spans="1:9" ht="15" thickBot="1">
-      <c r="A18" s="34" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="35"/>
-      <c r="C18" s="35"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-    </row>
-    <row r="19" spans="1:9" ht="15" thickBot="1">
-      <c r="A19" s="28" t="s">
-        <v>1</v>
-      </c>
-      <c r="B19" s="29" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="8">
-        <v>46086</v>
-      </c>
-      <c r="B20" s="31">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="16">
-        <v>46087</v>
-      </c>
-      <c r="B21" s="32">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="16">
-        <v>46093</v>
-      </c>
-      <c r="B22" s="32">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="16">
-        <v>46095</v>
-      </c>
-      <c r="B23" s="32">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="16">
-        <v>46100</v>
-      </c>
-      <c r="B24" s="32">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="16">
-        <v>46101</v>
-      </c>
-      <c r="B25" s="32" t="s">
-        <v>18</v>
-      </c>
-      <c r="C25" s="30" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" s="16">
-        <v>46107</v>
-      </c>
-      <c r="B26" s="32">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" ht="15" thickBot="1">
-      <c r="A27" s="12">
-        <v>46108</v>
-      </c>
-      <c r="B27" s="33" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" s="30" t="s">
-        <v>19</v>
-      </c>
-    </row>
+    <row r="17" ht="15"/>
+    <row r="18" ht="15"/>
+    <row r="19" ht="15"/>
+    <row r="20" ht="15"/>
+    <row r="21" ht="15"/>
+    <row r="22" ht="15"/>
+    <row r="23" ht="15"/>
+    <row r="24" ht="15"/>
+    <row r="25" ht="15"/>
+    <row r="26" ht="15"/>
+    <row r="27" ht="15"/>
+    <row r="28" ht="15"/>
+    <row r="29" ht="15"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A18:I18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
problem mit adaptivem radius bei analyseGlatt gehabt -> auf statischen radius geändert; probleme mit werten, der Grav-Algorithmus stimmt nicht!
</commit_message>
<xml_diff>
--- a/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
+++ b/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29930"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30002"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0EE37BE-6C99-439D-BD6D-6D41DB675F3C}"/>
+  <xr:revisionPtr revIDLastSave="50" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA0BCC1E-0463-4064-8B94-B24F07B0E737}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16305" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -202,7 +202,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -505,11 +505,69 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -533,7 +591,6 @@
     <xf numFmtId="16" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="21" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="21" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -560,19 +617,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="16" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="21" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="21" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="46" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="20" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="21" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="21" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="3" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -913,7 +968,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:S36"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="5" max="5" width="66.42578125" bestFit="1" customWidth="1"/>
@@ -921,17 +976,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="43" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="44"/>
-      <c r="C1" s="44"/>
-      <c r="D1" s="44"/>
-      <c r="E1" s="44"/>
-      <c r="F1" s="44"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="44"/>
-      <c r="I1" s="44"/>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
@@ -949,45 +1004,45 @@
       <c r="K2" s="2"/>
     </row>
     <row r="3" spans="1:19" ht="27.75">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="C3" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="D3" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="E3" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="26" t="s">
+      <c r="F3" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="26" t="s">
+      <c r="G3" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="26" t="s">
+      <c r="H3" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="27" t="s">
+      <c r="I3" s="26" t="s">
         <v>9</v>
       </c>
       <c r="J3" s="2"/>
-      <c r="K3" s="36" t="s">
+      <c r="K3" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="L3" s="37"/>
-      <c r="M3" s="37"/>
-      <c r="N3" s="37"/>
-      <c r="O3" s="37"/>
-      <c r="P3" s="37"/>
-      <c r="Q3" s="37"/>
-      <c r="R3" s="37"/>
-      <c r="S3" s="37"/>
+      <c r="L3" s="34"/>
+      <c r="M3" s="34"/>
+      <c r="N3" s="34"/>
+      <c r="O3" s="34"/>
+      <c r="P3" s="34"/>
+      <c r="Q3" s="34"/>
+      <c r="R3" s="34"/>
+      <c r="S3" s="34"/>
     </row>
     <row r="4" spans="1:19" ht="15">
       <c r="A4" s="20">
@@ -1020,10 +1075,10 @@
         <v>0.36805555555555552</v>
       </c>
       <c r="J4" s="2"/>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="L4" s="29" t="s">
+      <c r="L4" s="28" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1061,7 +1116,7 @@
       <c r="K5" s="8">
         <v>46086</v>
       </c>
-      <c r="L5" s="31">
+      <c r="L5" s="30">
         <v>55</v>
       </c>
     </row>
@@ -1099,7 +1154,7 @@
       <c r="K6" s="16">
         <v>46087</v>
       </c>
-      <c r="L6" s="32">
+      <c r="L6" s="31">
         <v>55</v>
       </c>
     </row>
@@ -1137,7 +1192,7 @@
       <c r="K7" s="16">
         <v>46093</v>
       </c>
-      <c r="L7" s="32">
+      <c r="L7" s="31">
         <v>55</v>
       </c>
     </row>
@@ -1175,7 +1230,7 @@
       <c r="K8" s="16">
         <v>46095</v>
       </c>
-      <c r="L8" s="32">
+      <c r="L8" s="31">
         <v>55</v>
       </c>
     </row>
@@ -1213,7 +1268,7 @@
       <c r="K9" s="16">
         <v>46100</v>
       </c>
-      <c r="L9" s="32">
+      <c r="L9" s="31">
         <v>55</v>
       </c>
     </row>
@@ -1251,10 +1306,10 @@
       <c r="K10" s="16">
         <v>46101</v>
       </c>
-      <c r="L10" s="32" t="s">
+      <c r="L10" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="M10" s="30" t="s">
+      <c r="M10" s="29" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1292,7 +1347,7 @@
       <c r="K11" s="16">
         <v>46107</v>
       </c>
-      <c r="L11" s="32">
+      <c r="L11" s="31">
         <v>55</v>
       </c>
     </row>
@@ -1330,10 +1385,10 @@
       <c r="K12" s="12">
         <v>46108</v>
       </c>
-      <c r="L12" s="33" t="s">
+      <c r="L12" s="32" t="s">
         <v>16</v>
       </c>
-      <c r="M12" s="30" t="s">
+      <c r="M12" s="29" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1341,35 +1396,35 @@
       <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="23">
+      <c r="I13" s="39">
         <f>SUM(I4:I12)</f>
         <v>2.7465277777777777</v>
       </c>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:19" ht="15">
-      <c r="A14" s="34">
-        <v>46117</v>
-      </c>
-      <c r="B14" s="35">
+      <c r="A14" s="35">
+        <v>46114</v>
+      </c>
+      <c r="B14" s="36">
         <v>0.38541666666666669</v>
       </c>
-      <c r="C14" s="38">
+      <c r="C14" s="36">
         <v>0.71527777777777779</v>
       </c>
-      <c r="D14" s="38">
+      <c r="D14" s="36">
         <v>0.3298611111111111</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="37" t="s">
         <v>20</v>
       </c>
-      <c r="F14" s="40">
+      <c r="F14" s="36">
         <v>0.5625</v>
       </c>
-      <c r="G14" s="38">
+      <c r="G14" s="36">
         <v>0.57986111111111116</v>
       </c>
-      <c r="H14" s="39">
+      <c r="H14" s="36">
         <v>1.7361111111111112E-2</v>
       </c>
       <c r="I14" s="38">
@@ -1378,68 +1433,297 @@
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:19" ht="15">
-      <c r="A15" s="34">
-        <v>46117</v>
-      </c>
-      <c r="B15" s="41">
+      <c r="A15" s="16">
+        <v>46114</v>
+      </c>
+      <c r="B15" s="3">
         <v>0.45833333333333331</v>
       </c>
-      <c r="C15" s="42">
+      <c r="C15" s="3">
         <v>5.5555555555555552E-2</v>
       </c>
-      <c r="D15" s="38">
+      <c r="D15" s="3">
         <v>9.7222222222222224E-2</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="3">
         <v>0</v>
       </c>
-      <c r="G15" s="22">
+      <c r="G15" s="3">
         <v>0</v>
       </c>
-      <c r="H15" s="38">
+      <c r="H15" s="3">
         <v>0</v>
       </c>
-      <c r="I15" s="38">
+      <c r="I15" s="17">
         <v>9.7222222222222224E-2</v>
       </c>
       <c r="J15" s="2"/>
       <c r="K15" s="2"/>
     </row>
     <row r="16" spans="1:19" ht="15">
-      <c r="A16" s="34">
-        <v>46118</v>
-      </c>
-      <c r="B16" s="35">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2" t="s">
+      <c r="A16" s="16">
+        <v>46115</v>
+      </c>
+      <c r="B16" s="3">
+        <v>0.40972222222222221</v>
+      </c>
+      <c r="C16" s="3">
+        <v>0.49652777777777779</v>
+      </c>
+      <c r="D16" s="3">
+        <v>8.6805555555555552E-2</v>
+      </c>
+      <c r="E16" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
+      <c r="F16" s="3">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3">
+        <v>0</v>
+      </c>
+      <c r="I16" s="17">
+        <v>8.6805555555555552E-2</v>
+      </c>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
     </row>
-    <row r="17" ht="15"/>
-    <row r="18" ht="15"/>
-    <row r="19" ht="15"/>
-    <row r="20" ht="15"/>
-    <row r="21" ht="15"/>
-    <row r="22" ht="15"/>
-    <row r="23" ht="15"/>
-    <row r="24" ht="15"/>
-    <row r="25" ht="15"/>
-    <row r="26" ht="15"/>
-    <row r="27" ht="15"/>
-    <row r="28" ht="15"/>
-    <row r="29" ht="15"/>
+    <row r="17" spans="1:9" ht="15">
+      <c r="A17" s="16">
+        <v>46121</v>
+      </c>
+      <c r="B17" s="3">
+        <v>0.3263888888888889</v>
+      </c>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="3">
+        <v>0.50694444444444442</v>
+      </c>
+      <c r="G17" s="3">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="H17" s="3">
+        <v>3.4722222222222224E-2</v>
+      </c>
+      <c r="I17" s="17"/>
+    </row>
+    <row r="18" spans="1:9" ht="15">
+      <c r="A18" s="16"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="17"/>
+    </row>
+    <row r="19" spans="1:9" ht="15">
+      <c r="A19" s="16"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="17"/>
+    </row>
+    <row r="20" spans="1:9" ht="15">
+      <c r="A20" s="16"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="17"/>
+    </row>
+    <row r="21" spans="1:9" ht="15">
+      <c r="A21" s="16"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="17"/>
+    </row>
+    <row r="22" spans="1:9" ht="15">
+      <c r="A22" s="16"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="17"/>
+    </row>
+    <row r="23" spans="1:9" ht="15">
+      <c r="A23" s="16"/>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="17"/>
+    </row>
+    <row r="24" spans="1:9" ht="15">
+      <c r="A24" s="16"/>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="17"/>
+    </row>
+    <row r="25" spans="1:9" ht="15">
+      <c r="A25" s="16"/>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="17"/>
+    </row>
+    <row r="26" spans="1:9" ht="15">
+      <c r="A26" s="16"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="17"/>
+    </row>
+    <row r="27" spans="1:9" ht="15">
+      <c r="A27" s="16"/>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="17"/>
+    </row>
+    <row r="28" spans="1:9" ht="15">
+      <c r="A28" s="16"/>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="17"/>
+    </row>
+    <row r="29" spans="1:9" ht="15">
+      <c r="A29" s="16"/>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="17"/>
+    </row>
+    <row r="30" spans="1:9" ht="15">
+      <c r="A30" s="16"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="17"/>
+    </row>
+    <row r="31" spans="1:9" ht="15">
+      <c r="A31" s="16"/>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="17"/>
+    </row>
+    <row r="32" spans="1:9" ht="15">
+      <c r="A32" s="16"/>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="17"/>
+    </row>
+    <row r="33" spans="1:9" ht="15">
+      <c r="A33" s="16"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="17"/>
+    </row>
+    <row r="34" spans="1:9" ht="15">
+      <c r="A34" s="16"/>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="17"/>
+    </row>
+    <row r="35" spans="1:9" ht="15">
+      <c r="A35" s="16"/>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="17"/>
+    </row>
+    <row r="36" spans="1:9" ht="15">
+      <c r="A36" s="16"/>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>

</xml_diff>

<commit_message>
to do: randbedingungen der kreise fixen
</commit_message>
<xml_diff>
--- a/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
+++ b/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA0BCC1E-0463-4064-8B94-B24F07B0E737}"/>
+  <xr:revisionPtr revIDLastSave="54" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E886DEF3-B537-4D12-BEFB-62DCD5A2F88C}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16305" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
   <si>
     <r>
       <t xml:space="preserve">März 2026: </t>
@@ -130,6 +130,9 @@
   </si>
   <si>
     <t>Code zur Speicherung der Analyse Daten geschrieben</t>
+  </si>
+  <si>
+    <t>Debugging - falsche Randbedingungen für die Mathematik des Codes</t>
   </si>
 </sst>
 </file>
@@ -1501,9 +1504,15 @@
       <c r="B17" s="3">
         <v>0.3263888888888889</v>
       </c>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="7"/>
+      <c r="C17" s="3">
+        <v>0.68402777777777779</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0.3576388888888889</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>23</v>
+      </c>
       <c r="F17" s="3">
         <v>0.50694444444444442</v>
       </c>
@@ -1513,7 +1522,9 @@
       <c r="H17" s="3">
         <v>3.4722222222222224E-2</v>
       </c>
-      <c r="I17" s="17"/>
+      <c r="I17" s="17">
+        <v>0.32291666666666669</v>
+      </c>
     </row>
     <row r="18" spans="1:9" ht="15">
       <c r="A18" s="16"/>

</xml_diff>

<commit_message>
erster durchbruch für punktauflager in Ordner CodeAblauf/Punktauflager; derzeitige probleme: wirken wenn punkte am rand, noch 'clamped' & wenn punkte in der mitte, ändert sich bei einer gewissen entfernung die krümmung und am rand wird die glasplatte wieder fast gerade
</commit_message>
<xml_diff>
--- a/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
+++ b/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30002"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30015"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="54" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E886DEF3-B537-4D12-BEFB-62DCD5A2F88C}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{729B8027-C141-4185-91E1-2D7FF5C10535}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16305" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="25">
   <si>
     <r>
       <t xml:space="preserve">März 2026: </t>
@@ -133,6 +133,9 @@
   </si>
   <si>
     <t>Debugging - falsche Randbedingungen für die Mathematik des Codes</t>
+  </si>
+  <si>
+    <t>Punktauflager implementiren</t>
   </si>
 </sst>
 </file>
@@ -1527,36 +1530,84 @@
       </c>
     </row>
     <row r="18" spans="1:9" ht="15">
-      <c r="A18" s="16"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="17"/>
+      <c r="A18" s="16">
+        <v>46128</v>
+      </c>
+      <c r="B18" s="3">
+        <v>0.36458333333333331</v>
+      </c>
+      <c r="C18" s="3">
+        <v>0.63888888888888884</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0.27430555555555558</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F18" s="3">
+        <v>0.51736111111111116</v>
+      </c>
+      <c r="G18" s="3">
+        <v>0.54513888888888884</v>
+      </c>
+      <c r="H18" s="3">
+        <v>2.7777777777777776E-2</v>
+      </c>
+      <c r="I18" s="17">
+        <v>0.24652777777777779</v>
+      </c>
     </row>
     <row r="19" spans="1:9" ht="15">
-      <c r="A19" s="16"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="17"/>
+      <c r="A19" s="16">
+        <v>46135</v>
+      </c>
+      <c r="B19" s="3">
+        <v>0.29166666666666669</v>
+      </c>
+      <c r="C19" s="3">
+        <v>0.3125</v>
+      </c>
+      <c r="D19" s="3">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="I19" s="17">
+        <v>2.0833333333333332E-2</v>
+      </c>
     </row>
     <row r="20" spans="1:9" ht="15">
-      <c r="A20" s="16"/>
-      <c r="B20" s="3"/>
+      <c r="A20" s="16">
+        <v>46135</v>
+      </c>
+      <c r="B20" s="3">
+        <v>0.3611111111111111</v>
+      </c>
       <c r="C20" s="3"/>
       <c r="D20" s="3"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
+      <c r="E20" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="3">
+        <v>0.50347222222222221</v>
+      </c>
+      <c r="G20" s="3">
+        <v>0.51736111111111116</v>
+      </c>
+      <c r="H20" s="3">
+        <v>1.3888888888888888E-2</v>
+      </c>
       <c r="I20" s="17"/>
     </row>
     <row r="21" spans="1:9" ht="15">

</xml_diff>

<commit_message>
ReissnerMindlin-Gleichung funktioniert nun, wirkt als funktioniert es als simply supported, einziges problem: rechnet noch in Meter, statt Millimeter
</commit_message>
<xml_diff>
--- a/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
+++ b/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{729B8027-C141-4185-91E1-2D7FF5C10535}"/>
+  <xr:revisionPtr revIDLastSave="87" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7978F26-3256-4632-A35D-408F45F071E0}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16305" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1594,8 +1594,12 @@
       <c r="B20" s="3">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
+      <c r="C20" s="3">
+        <v>0.75</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0.3888888888888889</v>
+      </c>
       <c r="E20" s="7" t="s">
         <v>24</v>
       </c>
@@ -1608,11 +1612,17 @@
       <c r="H20" s="3">
         <v>1.3888888888888888E-2</v>
       </c>
-      <c r="I20" s="17"/>
+      <c r="I20" s="17">
+        <v>0.375</v>
+      </c>
     </row>
     <row r="21" spans="1:9" ht="15">
-      <c r="A21" s="16"/>
-      <c r="B21" s="3"/>
+      <c r="A21" s="16">
+        <v>46136</v>
+      </c>
+      <c r="B21" s="3">
+        <v>0.41666666666666669</v>
+      </c>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="7"/>

</xml_diff>

<commit_message>
reissnerMindlin arbeitet zwar noch mit Meter, aber die simulation sieht nun super aus
</commit_message>
<xml_diff>
--- a/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
+++ b/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="87" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7978F26-3256-4632-A35D-408F45F071E0}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20291515-2ECA-45E9-9425-E979D17B0645}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16305" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1626,9 +1626,15 @@
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
       <c r="E21" s="7"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
+      <c r="F21" s="3">
+        <v>0.55902777777777779</v>
+      </c>
+      <c r="G21" s="3">
+        <v>0.59375</v>
+      </c>
+      <c r="H21" s="3">
+        <v>3.4722222222222224E-2</v>
+      </c>
       <c r="I21" s="17"/>
     </row>
     <row r="22" spans="1:9" ht="15">

</xml_diff>

<commit_message>
einiges in alteFiles verschoben; ziel jetzt: reissner mindlin von meter in millimeter umschreiben
</commit_message>
<xml_diff>
--- a/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
+++ b/Stunden+Kilometer Praktikum Anna Sonnleitner.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30015"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30023"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DE82BCE8-6750-4C1D-A7B4-F26B51045CB0}"/>
+  <xr:revisionPtr revIDLastSave="163" documentId="11_7CAF4A10D76DD5A139FB0C4AE06A9885A69E191F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8EB47AE5-52E5-4DE9-BC48-A5724860EBFD}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="16305" windowHeight="8250" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="29">
   <si>
     <r>
       <t xml:space="preserve">März 2026: </t>
@@ -123,6 +123,25 @@
     <t>Zwischenergebnis - MÄRZ</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Liberation Sans"/>
+      </rPr>
+      <t xml:space="preserve">April 2026: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Liberation Sans"/>
+      </rPr>
+      <t>Anna Sonnleitner (Fahrten nach Waidhofen/Ybbs  - Fa. SoftSolution)</t>
+    </r>
+  </si>
+  <si>
     <t>Erneut neues Konzept betreffend Auflagepunkte</t>
   </si>
   <si>
@@ -139,13 +158,19 @@
   </si>
   <si>
     <t>Reissner-Mindlin-Gleichung simulieren</t>
+  </si>
+  <si>
+    <t>Einkommenssteuerausgleich gemacht</t>
+  </si>
+  <si>
+    <t>Zwischenergebnis - APRIL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,6 +215,11 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Liberation Sans"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -211,7 +241,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="26">
+  <borders count="48">
     <border>
       <left/>
       <right/>
@@ -548,14 +578,275 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
-        <color rgb="FF000000"/>
-      </top>
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
       </bottom>
       <diagonal/>
     </border>
@@ -563,20 +854,37 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -634,15 +942,46 @@
     </xf>
     <xf numFmtId="16" fontId="2" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="21" fontId="2" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="21" fontId="2" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="46" fontId="3" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
+    <xf numFmtId="21" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="21" fontId="2" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="46" fontId="3" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -982,20 +1321,21 @@
   <cols>
     <col min="5" max="5" width="66.42578125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11.42578125" customWidth="1"/>
+    <col min="9" max="9" width="12.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="40" t="s">
+      <c r="A1" s="60" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="41"/>
-      <c r="C1" s="41"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="41"/>
-      <c r="F1" s="41"/>
-      <c r="G1" s="41"/>
-      <c r="H1" s="41"/>
-      <c r="I1" s="41"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
+      <c r="F1" s="61"/>
+      <c r="G1" s="61"/>
+      <c r="H1" s="61"/>
+      <c r="I1" s="61"/>
       <c r="J1" s="2"/>
       <c r="K1" s="2"/>
     </row>
@@ -1114,7 +1454,7 @@
         <v>0.5625</v>
       </c>
       <c r="H5" s="3">
-        <f t="shared" ref="H5:H12" si="0">G5-F5</f>
+        <f t="shared" ref="H5:H23" si="0">G5-F5</f>
         <v>2.083333333333337E-2</v>
       </c>
       <c r="I5" s="17">
@@ -1405,11 +1745,23 @@
       <c r="A13" t="s">
         <v>19</v>
       </c>
-      <c r="I13" s="39">
+      <c r="D13" s="48"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="54">
         <f>SUM(I4:I12)</f>
         <v>2.7465277777777777</v>
       </c>
       <c r="J13" s="2"/>
+      <c r="K13" s="65" t="s">
+        <v>20</v>
+      </c>
+      <c r="L13" s="34"/>
+      <c r="M13" s="34"/>
+      <c r="N13" s="66"/>
+      <c r="O13" s="66"/>
+      <c r="P13" s="66"/>
+      <c r="Q13" s="66"/>
+      <c r="R13" s="66"/>
     </row>
     <row r="14" spans="1:19" ht="15">
       <c r="A14" s="35">
@@ -1418,28 +1770,37 @@
       <c r="B14" s="36">
         <v>0.38541666666666669</v>
       </c>
-      <c r="C14" s="36">
+      <c r="C14" s="37">
         <v>0.71527777777777779</v>
       </c>
-      <c r="D14" s="36">
+      <c r="D14" s="53">
+        <f>C14-B14</f>
         <v>0.3298611111111111</v>
       </c>
-      <c r="E14" s="37" t="s">
-        <v>20</v>
+      <c r="E14" s="44" t="s">
+        <v>21</v>
       </c>
       <c r="F14" s="36">
         <v>0.5625</v>
       </c>
-      <c r="G14" s="36">
+      <c r="G14" s="37">
         <v>0.57986111111111116</v>
       </c>
-      <c r="H14" s="36">
-        <v>1.7361111111111112E-2</v>
-      </c>
-      <c r="I14" s="38">
-        <v>0.3125</v>
+      <c r="H14" s="53">
+        <f t="shared" si="0"/>
+        <v>1.736111111111116E-2</v>
+      </c>
+      <c r="I14" s="56">
+        <f>C14-B14-H14</f>
+        <v>0.31249999999999994</v>
       </c>
       <c r="J14" s="2"/>
+      <c r="K14" s="8">
+        <v>46114</v>
+      </c>
+      <c r="L14" s="30" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="15" spans="1:19" ht="15">
       <c r="A15" s="16">
@@ -1448,29 +1809,35 @@
       <c r="B15" s="3">
         <v>0.45833333333333331</v>
       </c>
-      <c r="C15" s="3">
+      <c r="C15" s="38">
         <v>5.5555555555555552E-2</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="40">
         <v>9.7222222222222224E-2</v>
       </c>
-      <c r="E15" s="7" t="s">
-        <v>21</v>
+      <c r="E15" s="45" t="s">
+        <v>22</v>
       </c>
       <c r="F15" s="3">
         <v>0</v>
       </c>
-      <c r="G15" s="3">
+      <c r="G15" s="38">
         <v>0</v>
       </c>
-      <c r="H15" s="3">
+      <c r="H15" s="40">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I15" s="17">
+      <c r="I15" s="57">
         <v>9.7222222222222224E-2</v>
       </c>
       <c r="J15" s="2"/>
-      <c r="K15" s="2"/>
+      <c r="K15" s="16">
+        <v>46114</v>
+      </c>
+      <c r="L15" s="31" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="16" spans="1:19" ht="15">
       <c r="A16" s="16">
@@ -1479,209 +1846,299 @@
       <c r="B16" s="3">
         <v>0.40972222222222221</v>
       </c>
-      <c r="C16" s="3">
+      <c r="C16" s="38">
         <v>0.49652777777777779</v>
       </c>
-      <c r="D16" s="3">
-        <v>8.6805555555555552E-2</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>22</v>
+      <c r="D16" s="40">
+        <f t="shared" ref="D15:D22" si="4">C16-B16</f>
+        <v>8.680555555555558E-2</v>
+      </c>
+      <c r="E16" s="46" t="s">
+        <v>23</v>
       </c>
       <c r="F16" s="3">
         <v>0</v>
       </c>
-      <c r="G16" s="3">
+      <c r="G16" s="38">
         <v>0</v>
       </c>
-      <c r="H16" s="3">
+      <c r="H16" s="40">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I16" s="17">
-        <v>8.6805555555555552E-2</v>
+      <c r="I16" s="57">
+        <f t="shared" ref="I15:I22" si="5">C16-B16-H16</f>
+        <v>8.680555555555558E-2</v>
       </c>
       <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-    </row>
-    <row r="17" spans="1:9" ht="15">
+      <c r="K16" s="16">
+        <v>46115</v>
+      </c>
+      <c r="L16" s="31">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" ht="15">
       <c r="A17" s="16">
         <v>46121</v>
       </c>
       <c r="B17" s="3">
         <v>0.3263888888888889</v>
       </c>
-      <c r="C17" s="3">
+      <c r="C17" s="38">
         <v>0.68402777777777779</v>
       </c>
-      <c r="D17" s="3">
+      <c r="D17" s="40">
+        <f t="shared" si="4"/>
         <v>0.3576388888888889</v>
       </c>
-      <c r="E17" s="7" t="s">
-        <v>23</v>
+      <c r="E17" s="45" t="s">
+        <v>24</v>
       </c>
       <c r="F17" s="3">
         <v>0.50694444444444442</v>
       </c>
-      <c r="G17" s="3">
+      <c r="G17" s="38">
         <v>0.54166666666666663</v>
       </c>
-      <c r="H17" s="3">
-        <v>3.4722222222222224E-2</v>
-      </c>
-      <c r="I17" s="17">
+      <c r="H17" s="40">
+        <f t="shared" si="0"/>
+        <v>3.472222222222221E-2</v>
+      </c>
+      <c r="I17" s="57">
+        <f t="shared" si="5"/>
         <v>0.32291666666666669</v>
       </c>
-    </row>
-    <row r="18" spans="1:9" ht="15">
+      <c r="K17" s="16">
+        <v>46121</v>
+      </c>
+      <c r="L17" s="31">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" ht="15">
       <c r="A18" s="16">
         <v>46128</v>
       </c>
       <c r="B18" s="3">
         <v>0.36458333333333331</v>
       </c>
-      <c r="C18" s="3">
+      <c r="C18" s="38">
         <v>0.63888888888888884</v>
       </c>
-      <c r="D18" s="3">
-        <v>0.27430555555555558</v>
-      </c>
-      <c r="E18" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F18" s="3">
+      <c r="D18" s="40">
+        <f t="shared" si="4"/>
+        <v>0.27430555555555552</v>
+      </c>
+      <c r="E18" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="F18" s="5">
         <v>0.51736111111111116</v>
       </c>
-      <c r="G18" s="3">
+      <c r="G18" s="39">
         <v>0.54513888888888884</v>
       </c>
-      <c r="H18" s="3">
-        <v>2.7777777777777776E-2</v>
-      </c>
-      <c r="I18" s="17">
-        <v>0.24652777777777779</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" ht="15">
+      <c r="H18" s="40">
+        <f t="shared" si="0"/>
+        <v>2.7777777777777679E-2</v>
+      </c>
+      <c r="I18" s="57">
+        <f t="shared" si="5"/>
+        <v>0.24652777777777785</v>
+      </c>
+      <c r="K18" s="16">
+        <v>46128</v>
+      </c>
+      <c r="L18" s="31">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" ht="15">
       <c r="A19" s="16">
         <v>46135</v>
       </c>
       <c r="B19" s="3">
         <v>0.29166666666666669</v>
       </c>
-      <c r="C19" s="3">
+      <c r="C19" s="38">
         <v>0.3125</v>
       </c>
-      <c r="D19" s="3">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F19" s="3" t="s">
+      <c r="D19" s="40">
+        <f t="shared" si="4"/>
+        <v>2.0833333333333315E-2</v>
+      </c>
+      <c r="E19" s="50" t="s">
+        <v>25</v>
+      </c>
+      <c r="F19" s="49">
+        <v>0</v>
+      </c>
+      <c r="G19" s="49">
+        <v>0</v>
+      </c>
+      <c r="H19" s="51">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="I19" s="57">
+        <f t="shared" si="5"/>
+        <v>2.0833333333333315E-2</v>
+      </c>
+      <c r="K19" s="16">
+        <v>46135</v>
+      </c>
+      <c r="L19" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="G19" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="I19" s="17">
-        <v>2.0833333333333332E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" ht="15">
+      <c r="M19" s="29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" ht="15">
       <c r="A20" s="16">
         <v>46135</v>
       </c>
       <c r="B20" s="3">
         <v>0.3611111111111111</v>
       </c>
-      <c r="C20" s="3">
+      <c r="C20" s="38">
         <v>0.75</v>
       </c>
-      <c r="D20" s="3">
+      <c r="D20" s="40">
+        <f t="shared" si="4"/>
         <v>0.3888888888888889</v>
       </c>
-      <c r="E20" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F20" s="3">
+      <c r="E20" s="45" t="s">
+        <v>25</v>
+      </c>
+      <c r="F20" s="6">
         <v>0.50347222222222221</v>
       </c>
-      <c r="G20" s="3">
+      <c r="G20" s="52">
         <v>0.51736111111111116</v>
       </c>
-      <c r="H20" s="3">
-        <v>1.3888888888888888E-2</v>
-      </c>
-      <c r="I20" s="17">
-        <v>0.375</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" ht="15">
+      <c r="H20" s="40">
+        <f t="shared" si="0"/>
+        <v>1.3888888888888951E-2</v>
+      </c>
+      <c r="I20" s="57">
+        <f t="shared" si="5"/>
+        <v>0.37499999999999994</v>
+      </c>
+      <c r="K20" s="16">
+        <v>46135</v>
+      </c>
+      <c r="L20" s="31">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" ht="15">
       <c r="A21" s="16">
         <v>46136</v>
       </c>
       <c r="B21" s="3">
         <v>0.41666666666666669</v>
       </c>
-      <c r="C21" s="3">
+      <c r="C21" s="38">
         <v>0.64583333333333337</v>
       </c>
-      <c r="D21" s="3">
-        <v>0.22916666666666666</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>25</v>
+      <c r="D21" s="40">
+        <f t="shared" si="4"/>
+        <v>0.22916666666666669</v>
+      </c>
+      <c r="E21" s="45" t="s">
+        <v>26</v>
       </c>
       <c r="F21" s="3">
         <v>0.55902777777777779</v>
       </c>
-      <c r="G21" s="3">
+      <c r="G21" s="38">
         <v>0.59375</v>
       </c>
-      <c r="H21" s="3">
-        <v>3.4722222222222224E-2</v>
-      </c>
-      <c r="I21" s="17">
-        <v>0.19444444444444445</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" ht="15">
-      <c r="A22" s="16"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="17"/>
-    </row>
-    <row r="23" spans="1:9" ht="15">
-      <c r="A23" s="16"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="17"/>
-    </row>
-    <row r="24" spans="1:9" ht="15">
-      <c r="A24" s="16"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
+      <c r="H21" s="40">
+        <f t="shared" si="0"/>
+        <v>3.472222222222221E-2</v>
+      </c>
+      <c r="I21" s="57">
+        <f t="shared" si="5"/>
+        <v>0.19444444444444448</v>
+      </c>
+      <c r="K21" s="18">
+        <v>46136</v>
+      </c>
+      <c r="L21" s="62" t="s">
+        <v>16</v>
+      </c>
+      <c r="M21" s="29" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" ht="15">
+      <c r="A22" s="18">
+        <v>46142</v>
+      </c>
+      <c r="B22" s="5">
+        <v>0.3263888888888889</v>
+      </c>
+      <c r="C22" s="39">
+        <v>0.72222222222222221</v>
+      </c>
+      <c r="D22" s="41">
+        <f t="shared" si="4"/>
+        <v>0.39583333333333331</v>
+      </c>
+      <c r="E22" s="47" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22" s="5">
+        <v>0.50694444444444442</v>
+      </c>
+      <c r="G22" s="39">
+        <v>0.53819444444444442</v>
+      </c>
+      <c r="H22" s="41">
+        <f t="shared" si="0"/>
+        <v>3.125E-2</v>
+      </c>
+      <c r="I22" s="58">
+        <f t="shared" si="5"/>
+        <v>0.36458333333333331</v>
+      </c>
+      <c r="K22" s="63">
+        <v>46142</v>
+      </c>
+      <c r="L22" s="64">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" ht="15">
+      <c r="A23" s="42" t="s">
+        <v>28</v>
+      </c>
+      <c r="B23" s="42"/>
+      <c r="C23" s="42"/>
+      <c r="D23" s="42"/>
+      <c r="E23" s="42"/>
+      <c r="F23" s="42"/>
+      <c r="G23" s="42"/>
+      <c r="H23" s="43"/>
+      <c r="I23" s="59">
+        <v>2.0208333333333335</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="15">
+      <c r="A24" s="20"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
       <c r="E24" s="7"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="17"/>
-    </row>
-    <row r="25" spans="1:9" ht="15">
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="21"/>
+    </row>
+    <row r="25" spans="1:13" ht="15">
       <c r="A25" s="16"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1692,7 +2149,7 @@
       <c r="H25" s="3"/>
       <c r="I25" s="17"/>
     </row>
-    <row r="26" spans="1:9" ht="15">
+    <row r="26" spans="1:13" ht="15">
       <c r="A26" s="16"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1703,7 +2160,7 @@
       <c r="H26" s="3"/>
       <c r="I26" s="17"/>
     </row>
-    <row r="27" spans="1:9" ht="15">
+    <row r="27" spans="1:13" ht="15">
       <c r="A27" s="16"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1714,7 +2171,7 @@
       <c r="H27" s="3"/>
       <c r="I27" s="17"/>
     </row>
-    <row r="28" spans="1:9" ht="15">
+    <row r="28" spans="1:13" ht="15">
       <c r="A28" s="16"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1725,7 +2182,7 @@
       <c r="H28" s="3"/>
       <c r="I28" s="17"/>
     </row>
-    <row r="29" spans="1:9" ht="15">
+    <row r="29" spans="1:13" ht="15">
       <c r="A29" s="16"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1736,7 +2193,7 @@
       <c r="H29" s="3"/>
       <c r="I29" s="17"/>
     </row>
-    <row r="30" spans="1:9" ht="15">
+    <row r="30" spans="1:13" ht="15">
       <c r="A30" s="16"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1747,7 +2204,7 @@
       <c r="H30" s="3"/>
       <c r="I30" s="17"/>
     </row>
-    <row r="31" spans="1:9" ht="15">
+    <row r="31" spans="1:13" ht="15">
       <c r="A31" s="16"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -1758,7 +2215,7 @@
       <c r="H31" s="3"/>
       <c r="I31" s="17"/>
     </row>
-    <row r="32" spans="1:9" ht="15">
+    <row r="32" spans="1:13" ht="15">
       <c r="A32" s="16"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>

</xml_diff>